<commit_message>
docs(apf3): RF37-CP02 probado en celular e informe final
</commit_message>
<xml_diff>
--- a/docs/anexos/Anexo_B_Fichas_CP_50_RF.xlsx
+++ b/docs/anexos/Anexo_B_Fichas_CP_50_RF.xlsx
@@ -43,7 +43,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -58,11 +58,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E2F3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -100,9 +95,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8119,7 +8111,7 @@
       </c>
       <c r="F149" s="4" t="inlineStr">
         <is>
-          <t>Celular Android con WhatsApp.</t>
+          <t>Celular Android (Chrome), estado de cuenta de Restaurante Sabor Norteño.</t>
         </is>
       </c>
       <c r="G149" s="4" t="inlineStr">
@@ -8132,9 +8124,9 @@
           <t>Se abre la hoja de compartir del celular con el PDF adjunto.</t>
         </is>
       </c>
-      <c r="I149" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente: el navegador de prueba no tiene hoja de compartir; se prueba en el celular del puesto.</t>
+      <c r="I149" s="4" t="inlineStr">
+        <is>
+          <t>Cumple. En un celular Android se abrió la hoja de compartir con el PDF EstadoCuenta adjunto (captura rf37_cp02).</t>
         </is>
       </c>
       <c r="J149" s="4" t="inlineStr">

</xml_diff>